<commit_message>
💡 Mejora formato de tabla en Streamlit para matriz de pruebas
</commit_message>
<xml_diff>
--- a/Outputs/matriz_pruebas.xlsx
+++ b/Outputs/matriz_pruebas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,17 +458,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Login exitoso</t>
+          <t>Acceso al flujo de transferencias</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Usuario válido y contraseña correcta</t>
+          <t>Feature Flag `LD_TRANSFER_INTERBANCARIA = true`</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Acceso concedido</t>
+          <t>El menú “Transferencias” es visible.</t>
         </is>
       </c>
     </row>
@@ -480,17 +480,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Login fallido</t>
+          <t>Acceso al flujo de transferencias</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Usuario inválido y contraseña errónea</t>
+          <t>Feature Flag `LD_TRANSFER_INTERBANCARIA = false`</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mensaje de error “Credenciales incorrectas”</t>
+          <t>El menú “Transferencias” no es visible.</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bloqueo de cuenta tras 3 intentos fallidos</t>
+          <t>Mostrar cuentas destino registradas</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Usuario válido y 3 contraseñas erróneas</t>
+          <t>Cuentas destino registradas</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Cuenta bloqueada y mensaje de error</t>
+          <t>Se muestran las cuentas destino registradas.</t>
         </is>
       </c>
     </row>
@@ -524,17 +524,149 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Registro de fecha y hora del último intento</t>
+          <t>Mensaje si no hay cuentas registradas</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Usuario válido y contraseña errónea</t>
+          <t>No hay cuentas registradas</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Fecha y hora del último intento registrado</t>
+          <t>Se muestra el mensaje “No tienes cuentas guardadas. Agrega una nueva cuenta destino.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Transferencia con monto válido</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Monto: $500.000</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Se muestra el resumen de la transferencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Transferencia con monto que excede el límite</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Monto: $1.500.000</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Se muestra el mensaje “El monto supera el límite permitido.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Confirmar transferencia exitosa</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Datos de transferencia válidos</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Se muestra el mensaje “Tu transferencia fue realizada con éxito.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Confirmar transferencia con error técnico</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Datos de transferencia válidos, pero error en el backend</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Se muestra el mensaje “No pudimos completar tu transferencia. Intenta más tarde.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Respuesta del backend con estado SUCCESS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Transferencia exitosa</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>El estado de la respuesta es SUCCESS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Respuesta del backend con estado ERROR</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Transferencia fallida</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>El estado de la respuesta es ERROR.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add .env.example and update .gitignore
</commit_message>
<xml_diff>
--- a/Outputs/matriz_pruebas.xlsx
+++ b/Outputs/matriz_pruebas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,17 +458,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Acceso al flujo de transferencias</t>
+          <t>Login exitoso</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Feature Flag `LD_TRANSFER_INTERBANCARIA = true`</t>
+          <t>Correo: usuario@ejemplo.com, Contraseña: contraseña123</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>El menú “Transferencias” es visible.</t>
+          <t>Redirige a /dashboard mostrando "Bienvenido/a nuevamente."</t>
         </is>
       </c>
     </row>
@@ -480,17 +480,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Acceso al flujo de transferencias</t>
+          <t>Login fallido - campos vacíos</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Feature Flag `LD_TRANSFER_INTERBANCARIA = false`</t>
+          <t>Correo: "", Contraseña: ""</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>El menú “Transferencias” no es visible.</t>
+          <t>Muestra "Por favor, completa todos los campos."</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mostrar cuentas destino registradas</t>
+          <t>Login fallido - correo inválido</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cuentas destino registradas</t>
+          <t>Correo: usuarioejemplo.com, Contraseña: contraseña123</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Se muestran las cuentas destino registradas.</t>
+          <t>Muestra "Correo electrónico inválido."</t>
         </is>
       </c>
     </row>
@@ -524,149 +524,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mensaje si no hay cuentas registradas</t>
+          <t>Login fallido - credenciales incorrectas</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>No hay cuentas registradas</t>
+          <t>Correo: usuario@ejemplo.com, Contraseña: incorrecta123</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Se muestra el mensaje “No tienes cuentas guardadas. Agrega una nueva cuenta destino.”</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>TC005</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Transferencia con monto válido</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Monto: $500.000</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Se muestra el resumen de la transferencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>TC006</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Transferencia con monto que excede el límite</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Monto: $1.500.000</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Se muestra el mensaje “El monto supera el límite permitido.”</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>TC007</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Confirmar transferencia exitosa</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Datos de transferencia válidos</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Se muestra el mensaje “Tu transferencia fue realizada con éxito.”</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>TC008</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Confirmar transferencia con error técnico</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Datos de transferencia válidos, pero error en el backend</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Se muestra el mensaje “No pudimos completar tu transferencia. Intenta más tarde.”</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>TC009</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Respuesta del backend con estado SUCCESS</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Transferencia exitosa</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>El estado de la respuesta es SUCCESS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>TC010</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Respuesta del backend con estado ERROR</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Transferencia fallida</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>El estado de la respuesta es ERROR.</t>
+          <t>Muestra "Credenciales incorrectas."</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Integrar Modal con Hannah QA Agent
- ✅ Configurar Doppler para archivos en src/ con variables seguras
- ✅ Crear hannah_modal_app.py para backend serverless en Modal
- ✅ Crear hannah_modal_client.py para conexión simplificada
- ✅ Modificar app_hannah_error_handling.py para usar Modal como backend
- ✅ Agregar scripts npm para ejecutar archivos en src/ con Doppler
- ✅ Desplegar Hannah a Modal Cloud exitosamente
- ✅ Conectar frontend Streamlit con backend Modal
- ✅ Agregar Modal a requirements.txt
- ✅ Crear archivos de prueba y configuración

Funcionalidades:
- Frontend: Streamlit local con interfaz moderna
- Backend: Modal serverless con IA de OpenAI
- Variables: Doppler secure para todas las configuraciones
- Scripts: npm run commands para ejecutar cualquier archivo en src/
</commit_message>
<xml_diff>
--- a/Outputs/matriz_pruebas.xlsx
+++ b/Outputs/matriz_pruebas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,17 +458,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Login exitoso</t>
+          <t>Registro exitoso</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Correo: usuario@ejemplo.com, Contraseña: contraseña123</t>
+          <t>Correo: usuario@ejemplo.com, Nombre: Juan, Contraseña: Contraseña123</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Redirige a /dashboard mostrando "Bienvenido/a nuevamente."</t>
+          <t>Usuario registrado correctamente</t>
         </is>
       </c>
     </row>
@@ -480,17 +480,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Login fallido - campos vacíos</t>
+          <t>Registro fallido - Correo existente</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Correo: "", Contraseña: ""</t>
+          <t>Correo: usuario@ejemplo.com, Nombre: Pedro, Contraseña: Contraseña456</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Muestra "Por favor, completa todos los campos."</t>
+          <t>Mensaje de error "El correo ya está registrado"</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Login fallido - correo inválido</t>
+          <t>Registro fallido - Contraseña débil</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Correo: usuarioejemplo.com, Contraseña: contraseña123</t>
+          <t>Correo: nuevo@ejemplo.com, Nombre: Ana, Contraseña: 123</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Muestra "Correo electrónico inválido."</t>
+          <t>Mensaje de error "La contraseña debe tener al menos 8 caracteres"</t>
         </is>
       </c>
     </row>
@@ -524,17 +524,39 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Login fallido - credenciales incorrectas</t>
+          <t>Registro fallido - Campos vacíos</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Correo: usuario@ejemplo.com, Contraseña: incorrecta123</t>
+          <t>Correo: , Nombre: , Contraseña:</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Muestra "Credenciales incorrectas."</t>
+          <t>Mensaje de error "Todos los campos son obligatorios"</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Registro fallido - Formato de correo inválido</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Correo: usuarioejemplo.com, Nombre: Luis, Contraseña: Contraseña789</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Mensaje de error "Formato de correo inválido"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Integración completa de Doppler, Modal y Axiom en Hannah QA Agent
</commit_message>
<xml_diff>
--- a/Outputs/matriz_pruebas.xlsx
+++ b/Outputs/matriz_pruebas.xlsx
@@ -480,17 +480,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Registro fallido - Correo existente</t>
+          <t>Registro fallido - correo ya existe</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Correo: usuario@ejemplo.com, Nombre: Pedro, Contraseña: Contraseña456</t>
+          <t>Correo: usuario@ejemplo.com, Nombre: Juan, Contraseña: Contraseña123</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mensaje de error "El correo ya está registrado"</t>
+          <t>Mensaje de error "El correo ya está en uso"</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Registro fallido - Contraseña débil</t>
+          <t>Registro fallido - contraseña débil</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mensaje de error "La contraseña debe tener al menos 8 caracteres"</t>
+          <t>Mensaje de error "La contraseña es demasiado débil"</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Registro fallido - Campos vacíos</t>
+          <t>Registro fallido - datos incompletos</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Correo: , Nombre: , Contraseña:</t>
+          <t>Correo: , Nombre: Juan, Contraseña: Contraseña123</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Registro fallido - Formato de correo inválido</t>
+          <t>Registro fallido - formato de correo inválido</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Correo: usuarioejemplo.com, Nombre: Luis, Contraseña: Contraseña789</t>
+          <t>Correo: usuario@ejemplo, Nombre: Juan, Contraseña: Contraseña123</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">

</xml_diff>

<commit_message>
Simplificación completa del proyecto: backend y frontend optimizados
- Backend: Reducido 30% de código (600+ líneas eliminadas)
  - Eliminados 6 archivos duplicados
  - Creado utils_axiom.py para logging centralizado
  - Simplificados app_hannah_error_handling.py y archivos relacionados
  - Mejorado hannah_modal_client.py (60% más simple)
  - Fallback automático a OpenAI si Modal no está disponible

- Frontend: Reducido 25% de código (63 líneas eliminadas)
  - Simplificados page.tsx, layout.tsx y globals.css
  - Eliminados 5 SVGs innecesarios
  - README actualizado con documentación específica

- Scripts bash para ejecutar todos los archivos .py
- COMANDOS_RAPIDOS.md con guía de uso
- Tests mejorados con mejor manejo de errores

Total: ~663 líneas reducidas, 11 archivos eliminados, 10 scripts bash creados
</commit_message>
<xml_diff>
--- a/Outputs/matriz_pruebas.xlsx
+++ b/Outputs/matriz_pruebas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,17 +458,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Registro exitoso</t>
+          <t>Login exitoso</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Correo: usuario@ejemplo.com, Nombre: Juan, Contraseña: Contraseña123</t>
+          <t>Correo electrónico y contraseña válidos</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Usuario registrado correctamente</t>
+          <t>Acceso concedido y redirección a la página principal</t>
         </is>
       </c>
     </row>
@@ -480,17 +480,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Registro fallido - correo ya existe</t>
+          <t>Login fallido</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Correo: usuario@ejemplo.com, Nombre: Juan, Contraseña: Contraseña123</t>
+          <t>Correo electrónico incorrecto y contraseña válida</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mensaje de error "El correo ya está en uso"</t>
+          <t>Mensaje de error indicando credenciales incorrectas</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Registro fallido - contraseña débil</t>
+          <t>Login fallido</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Correo: nuevo@ejemplo.com, Nombre: Ana, Contraseña: 123</t>
+          <t>Correo electrónico válido y contraseña incorrecta</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mensaje de error "La contraseña es demasiado débil"</t>
+          <t>Mensaje de error indicando credenciales incorrectas</t>
         </is>
       </c>
     </row>
@@ -524,39 +524,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Registro fallido - datos incompletos</t>
+          <t>Login fallido</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Correo: , Nombre: Juan, Contraseña: Contraseña123</t>
+          <t>Correo electrónico y contraseña vacíos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mensaje de error "Todos los campos son obligatorios"</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>TC005</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Registro fallido - formato de correo inválido</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Correo: usuario@ejemplo, Nombre: Juan, Contraseña: Contraseña123</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Mensaje de error "Formato de correo inválido"</t>
+          <t>Mensaje de error indicando que los campos son obligatorios</t>
         </is>
       </c>
     </row>

</xml_diff>